<commit_message>
I still need to test MOSFET circuits in Ltspice but I cleaned up the v2 Schematic and starting routing v2 PCB
</commit_message>
<xml_diff>
--- a/Documentation/Contributions/TimeReport_CarterKreis.xlsx
+++ b/Documentation/Contributions/TimeReport_CarterKreis.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="67">
   <si>
     <t xml:space="preserve">Name:</t>
   </si>
@@ -212,6 +212,15 @@
   </si>
   <si>
     <t xml:space="preserve">I ordered the PCB!! … there is so many changes I want to make but I also just wanted to order it but without the revisions it was more expensive but now we at least will have a board. Welp, either way I will solve the NPK (again unfortunately) next and then after that get onto PCB V2 and then 3D modeling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Release Candidate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Researched more into implemented PWM driven MOSFET circuit to replace 5V relays. Tested liquid pumps to see what voltages were actually needed to power them and learned that 12V is wayyy overkill. I also finished schematic for new MOSFET circuits and will Ltspice next</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I still need to test MOSFET circuits in Ltspice but I cleaned up the v2 Schematic and starting routing v2 PCB</t>
   </si>
 </sst>
 </file>
@@ -605,7 +614,7 @@
       </c>
       <c r="E1" s="4" t="n">
         <f aca="false">SUM(E4:E199)</f>
-        <v>4.79027777777778</v>
+        <v>4.95347222222222</v>
       </c>
       <c r="F1" s="5"/>
     </row>
@@ -1575,26 +1584,46 @@
       </c>
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="16"/>
-      <c r="B49" s="7"/>
-      <c r="C49" s="17"/>
-      <c r="D49" s="17"/>
+      <c r="A49" s="16" t="n">
+        <v>46079</v>
+      </c>
+      <c r="B49" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C49" s="17" t="n">
+        <v>0.496527777777778</v>
+      </c>
+      <c r="D49" s="17" t="n">
+        <v>0.597222222222222</v>
+      </c>
       <c r="E49" s="9" t="n">
         <f aca="false">D49-C49</f>
-        <v>0</v>
-      </c>
-      <c r="F49" s="10"/>
+        <v>0.100694444444444</v>
+      </c>
+      <c r="F49" s="10" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="16"/>
-      <c r="B50" s="7"/>
-      <c r="C50" s="17"/>
-      <c r="D50" s="17"/>
+      <c r="A50" s="16" t="n">
+        <v>46079</v>
+      </c>
+      <c r="B50" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C50" s="17" t="n">
+        <v>0.763888888888889</v>
+      </c>
+      <c r="D50" s="17" t="n">
+        <v>0.826388888888889</v>
+      </c>
       <c r="E50" s="9" t="n">
         <f aca="false">D50-C50</f>
-        <v>0</v>
-      </c>
-      <c r="F50" s="10"/>
+        <v>0.0625</v>
+      </c>
+      <c r="F50" s="10" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="16"/>

</xml_diff>

<commit_message>
Routed v2 PCB some more. Finished routing power sources, Buck Converter, MOSFET circuits, and most of RS485 Transceiver. I forgot about KiCad but will not next time I get a big chunk of time
</commit_message>
<xml_diff>
--- a/Documentation/Contributions/TimeReport_CarterKreis.xlsx
+++ b/Documentation/Contributions/TimeReport_CarterKreis.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="68">
   <si>
     <t xml:space="preserve">Name:</t>
   </si>
@@ -221,6 +221,9 @@
   </si>
   <si>
     <t xml:space="preserve">I still need to test MOSFET circuits in Ltspice but I cleaned up the v2 Schematic and starting routing v2 PCB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Routed v2 PCB some more. Finished routing power sources, Buck Converter, MOSFET circuits, and most of RS485 Transceiver. I forgot about KiCad but will not next time I get a big chunk of time</t>
   </si>
 </sst>
 </file>
@@ -614,7 +617,7 @@
       </c>
       <c r="E1" s="4" t="n">
         <f aca="false">SUM(E4:E199)</f>
-        <v>4.95347222222222</v>
+        <v>5.00208333333333</v>
       </c>
       <c r="F1" s="5"/>
     </row>
@@ -1626,15 +1629,25 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="16"/>
-      <c r="B51" s="7"/>
-      <c r="C51" s="17"/>
-      <c r="D51" s="17"/>
+      <c r="A51" s="16" t="n">
+        <v>46081</v>
+      </c>
+      <c r="B51" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C51" s="17" t="n">
+        <v>0.763888888888889</v>
+      </c>
+      <c r="D51" s="17" t="n">
+        <v>0.8125</v>
+      </c>
       <c r="E51" s="9" t="n">
         <f aca="false">D51-C51</f>
-        <v>0</v>
-      </c>
-      <c r="F51" s="10"/>
+        <v>0.0486111111111111</v>
+      </c>
+      <c r="F51" s="10" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="16"/>

</xml_diff>

<commit_message>
Meeting with Tyler. Fully finished routing MOSFET circuits, RS485 Transceiver, and some of ADC circuits. Still need to test MOSFET circuits in Ltspice, but placed most of overall PCB into a small edge cut square that is 2.5”x2.5” which is 50% smaller and cheaper.
</commit_message>
<xml_diff>
--- a/Documentation/Contributions/TimeReport_CarterKreis.xlsx
+++ b/Documentation/Contributions/TimeReport_CarterKreis.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="69">
   <si>
     <t xml:space="preserve">Name:</t>
   </si>
@@ -223,7 +223,10 @@
     <t xml:space="preserve">I still need to test MOSFET circuits in Ltspice but I cleaned up the v2 Schematic and starting routing v2 PCB</t>
   </si>
   <si>
-    <t xml:space="preserve">Routed v2 PCB some more. Finished routing power sources, Buck Converter, MOSFET circuits, and most of RS485 Transceiver. I forgot about KiCad but will not next time I get a big chunk of time</t>
+    <t xml:space="preserve">Routed v2 PCB some more. Finished routing power sources, Buck Converter, MOSFET circuits, and most of RS485 Transceiver. I forgot about Ltspice but will not next time I get a big chunk of time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meeting with Tyler. Fully finished routing MOSFET circuits, RS485 Transceiver, and some of ADC circuits. Still need to test MOSFET circuits in Ltspice, but placed most of overall PCB into a small edge cut square that is 2.5”x2.5” which is 50% smaller and cheaper.</t>
   </si>
 </sst>
 </file>
@@ -617,7 +620,7 @@
       </c>
       <c r="E1" s="4" t="n">
         <f aca="false">SUM(E4:E199)</f>
-        <v>5.00208333333333</v>
+        <v>5.08541666666667</v>
       </c>
       <c r="F1" s="5"/>
     </row>
@@ -1650,15 +1653,25 @@
       </c>
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="16"/>
-      <c r="B52" s="7"/>
-      <c r="C52" s="17"/>
-      <c r="D52" s="17"/>
+      <c r="A52" s="16" t="n">
+        <v>46083</v>
+      </c>
+      <c r="B52" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C52" s="17" t="n">
+        <v>0.420138888888889</v>
+      </c>
+      <c r="D52" s="17" t="n">
+        <v>0.503472222222222</v>
+      </c>
       <c r="E52" s="9" t="n">
         <f aca="false">D52-C52</f>
-        <v>0</v>
-      </c>
-      <c r="F52" s="10"/>
+        <v>0.0833333333333333</v>
+      </c>
+      <c r="F52" s="10" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="16"/>

</xml_diff>

<commit_message>
Finished routing everything. Adding silkscreens and double checking details. Next I will test in Ltspice. Hopefully, place JLC order by tonight or tomorrow
</commit_message>
<xml_diff>
--- a/Documentation/Contributions/TimeReport_CarterKreis.xlsx
+++ b/Documentation/Contributions/TimeReport_CarterKreis.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="70">
   <si>
     <t xml:space="preserve">Name:</t>
   </si>
@@ -227,6 +227,9 @@
   </si>
   <si>
     <t xml:space="preserve">Meeting with Tyler. Fully finished routing MOSFET circuits, RS485 Transceiver, and some of ADC circuits. Still need to test MOSFET circuits in Ltspice, but placed most of overall PCB into a small edge cut square that is 2.5”x2.5” which is 50% smaller and cheaper.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finished routing everything. Adding silkscreens and double checking details. Next I will test in Ltspice. Hopefully, place JLC order by tonight or tomorrow</t>
   </si>
 </sst>
 </file>
@@ -620,7 +623,7 @@
       </c>
       <c r="E1" s="4" t="n">
         <f aca="false">SUM(E4:E199)</f>
-        <v>5.08541666666667</v>
+        <v>5.22083333333333</v>
       </c>
       <c r="F1" s="5"/>
     </row>
@@ -1674,15 +1677,25 @@
       </c>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="16"/>
-      <c r="B53" s="7"/>
-      <c r="C53" s="17"/>
-      <c r="D53" s="17"/>
+      <c r="A53" s="16" t="n">
+        <v>46083</v>
+      </c>
+      <c r="B53" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C53" s="17" t="n">
+        <v>0.572916666666667</v>
+      </c>
+      <c r="D53" s="17" t="n">
+        <v>0.708333333333333</v>
+      </c>
       <c r="E53" s="9" t="n">
         <f aca="false">D53-C53</f>
-        <v>0</v>
-      </c>
-      <c r="F53" s="10"/>
+        <v>0.135416666666667</v>
+      </c>
+      <c r="F53" s="10" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="16"/>

</xml_diff>

<commit_message>
Ordered PCB v2 after verifying MOSFET PWM circuits in Ltspicegit add . It was definitely cheaper but still just over 0 for all 5 to be assembled with SMT parts. Next I’ll work on “solving” the NPK so we can implement it to the entire system.
</commit_message>
<xml_diff>
--- a/Documentation/Contributions/TimeReport_CarterKreis.xlsx
+++ b/Documentation/Contributions/TimeReport_CarterKreis.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="71">
   <si>
     <t xml:space="preserve">Name:</t>
   </si>
@@ -230,6 +230,9 @@
   </si>
   <si>
     <t xml:space="preserve">Finished routing everything. Adding silkscreens and double checking details. Next I will test in Ltspice. Hopefully, place JLC order by tonight or tomorrow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ordered PCB v2 after verifying MOSFET PWM circuits in Ltspice!! It was definitely cheaper but still just over $50 for all 5 to be assembled with SMT parts. Next I’ll work on “solving” the NPK so we can implement it to the entire system.</t>
   </si>
 </sst>
 </file>
@@ -623,7 +626,7 @@
       </c>
       <c r="E1" s="4" t="n">
         <f aca="false">SUM(E4:E199)</f>
-        <v>5.22083333333333</v>
+        <v>5.33541666666667</v>
       </c>
       <c r="F1" s="5"/>
     </row>
@@ -1698,15 +1701,25 @@
       </c>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="16"/>
-      <c r="B54" s="7"/>
-      <c r="C54" s="17"/>
-      <c r="D54" s="17"/>
+      <c r="A54" s="16" t="n">
+        <v>46084</v>
+      </c>
+      <c r="B54" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C54" s="17" t="n">
+        <v>0.479166666666667</v>
+      </c>
+      <c r="D54" s="17" t="n">
+        <v>0.59375</v>
+      </c>
       <c r="E54" s="9" t="n">
         <f aca="false">D54-C54</f>
-        <v>0</v>
-      </c>
-      <c r="F54" s="10"/>
+        <v>0.114583333333333</v>
+      </c>
+      <c r="F54" s="10" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="16"/>

</xml_diff>

<commit_message>
Updating Timesheet ... yeah I got no idea why I didn't merge my latest timesheet into main lol
</commit_message>
<xml_diff>
--- a/Documentation/Contributions/TimeReport_CarterKreis.xlsx
+++ b/Documentation/Contributions/TimeReport_CarterKreis.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="75">
   <si>
     <t xml:space="preserve">Name:</t>
   </si>
@@ -293,6 +293,9 @@
   </si>
   <si>
     <t xml:space="preserve">Worked on soldering PCBv1 some more. Most of the testing pins are in and all the screw terminals are in. Next will be the two SMD parts and any of the more difficult parts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Worked on Documentation over break so that’s why the long gap, but today I helped finalize the 3D modeling for the Liquid Housing, PCB Housing, and PCB Lid by adding connector pins. I also spent some time helping Nico test the entire projects connectivity but we had issues connected to WiFi for HTTP communication.</t>
   </si>
 </sst>
 </file>
@@ -414,7 +417,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -488,6 +491,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -698,7 +705,7 @@
       </c>
       <c r="E1" s="4" t="n">
         <f aca="false">SUM(E4:E199)</f>
-        <v>5.65486111111111</v>
+        <v>5.77638888888889</v>
       </c>
       <c r="F1" s="5"/>
     </row>
@@ -1855,17 +1862,28 @@
       <c r="F57" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="G57" s="0"/>
+      <c r="G57" s="19"/>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="16"/>
-      <c r="B58" s="7"/>
-      <c r="C58" s="17"/>
-      <c r="D58" s="17"/>
+      <c r="A58" s="16" t="n">
+        <v>46105</v>
+      </c>
+      <c r="B58" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C58" s="17" t="n">
+        <v>0.524305555555556</v>
+      </c>
+      <c r="D58" s="17" t="n">
+        <v>0.645833333333333</v>
+      </c>
       <c r="E58" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F58" s="0"/>
+        <f aca="false">D58-C58</f>
+        <v>0.121527777777778</v>
+      </c>
+      <c r="F58" s="19" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="16"/>

</xml_diff>

<commit_message>
Updated Timesheet for 3D modeling
</commit_message>
<xml_diff>
--- a/Documentation/Contributions/TimeReport_CarterKreis.xlsx
+++ b/Documentation/Contributions/TimeReport_CarterKreis.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="76">
   <si>
     <t xml:space="preserve">Name:</t>
   </si>
@@ -296,6 +296,9 @@
   </si>
   <si>
     <t xml:space="preserve">Worked on Documentation over break so that’s why the long gap, but today I helped finalize the 3D modeling for the Liquid Housing, PCB Housing, and PCB Lid by adding connector pins. I also spent some time helping Nico test the entire projects connectivity but we had issues connected to WiFi for HTTP communication.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Added the connection holes for the Moisture Sensor and NPK but I can get part of the Moisture Sensor sketch to be fully defined</t>
   </si>
 </sst>
 </file>
@@ -705,7 +708,7 @@
       </c>
       <c r="E1" s="4" t="n">
         <f aca="false">SUM(E4:E199)</f>
-        <v>5.77638888888889</v>
+        <v>5.87013888888889</v>
       </c>
       <c r="F1" s="5"/>
     </row>
@@ -1886,15 +1889,25 @@
       </c>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="16"/>
-      <c r="B59" s="7"/>
-      <c r="C59" s="17"/>
-      <c r="D59" s="17"/>
+      <c r="A59" s="16" t="n">
+        <v>46107</v>
+      </c>
+      <c r="B59" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C59" s="17" t="n">
+        <v>0.510416666666667</v>
+      </c>
+      <c r="D59" s="17" t="n">
+        <v>0.604166666666667</v>
+      </c>
       <c r="E59" s="9" t="n">
         <f aca="false">D59-C59</f>
-        <v>0</v>
-      </c>
-      <c r="F59" s="10"/>
+        <v>0.09375</v>
+      </c>
+      <c r="F59" s="10" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="16"/>

</xml_diff>

<commit_message>
Updated Timesheet and Release Candidate meeting w/ Tyler
</commit_message>
<xml_diff>
--- a/Documentation/Contributions/TimeReport_CarterKreis.xlsx
+++ b/Documentation/Contributions/TimeReport_CarterKreis.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="80">
   <si>
     <t xml:space="preserve">Name:</t>
   </si>
@@ -308,6 +308,9 @@
   </si>
   <si>
     <t xml:space="preserve">Drilled holes for fertilizer and water pump tubes and power cords. Soldered wire extensions for Lamp then heat-shrinked and taped them. Attempted to desolder Light Sensor pins on PCB to swap for Female Headers but destroyed PCB pad. For Tyler Demo tomorrow, I will make some small external circuitry but I will help solder a new board by early next week. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Since we burned the Light Sensor PCB Pad, I breadboarded a quick solution. Then we demo’d our project to Tyler who said everything was good.</t>
   </si>
 </sst>
 </file>
@@ -717,7 +720,7 @@
       </c>
       <c r="E1" s="4" t="n">
         <f aca="false">SUM(E4:E199)</f>
-        <v>6.29027777777778</v>
+        <v>6.34583333333333</v>
       </c>
       <c r="F1" s="5"/>
     </row>
@@ -1982,15 +1985,25 @@
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="16"/>
-      <c r="B63" s="7"/>
-      <c r="C63" s="17"/>
-      <c r="D63" s="17"/>
+      <c r="A63" s="16" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B63" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C63" s="17" t="n">
+        <v>0.427083333333333</v>
+      </c>
+      <c r="D63" s="17" t="n">
+        <v>0.482638888888889</v>
+      </c>
       <c r="E63" s="9" t="n">
         <f aca="false">D63-C63</f>
-        <v>0</v>
-      </c>
-      <c r="F63" s="10"/>
+        <v>0.0555555555555556</v>
+      </c>
+      <c r="F63" s="10" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="16"/>

</xml_diff>